<commit_message>
Apply sprint 3 review fixes and separate BUG-014
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -25,30 +25,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="B32" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Запропонований кейс: ще не внесений до test-cases.xlsx і не прорецензований.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="215">
   <si>
     <t xml:space="preserve">Run</t>
   </si>
@@ -266,262 +244,265 @@
     <t xml:space="preserve">TC-026</t>
   </si>
   <si>
+    <t xml:space="preserve">BUG-009, BUG-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фактично: Кроки 13–14: пароль «Abcde1!» (7 символів) відхилено, але повідомлення «Password must be minimal 6 characters long.» називає межу 6 символів, що суперечить правилу «Be at least 8 characters long» на цій самій сторінці (F-10) — BUG-009. Повідомлення виведено в блоці над кнопкою «Register» (під переліком правил та індикатором надійності), а не безпосередньо під полем «Password» (GUI-50) — BUG-014. Дефект: BUG-009, BUG-014.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рядок довжиною рівно 50 символів (перевірено програмно). Крок 7: форма замінилась на «Thanks for your message! We will contact you shortly.» (клас alert-success) над блоком футера; помилок немає. Це реальне надсилання на demo з тестовим email example.com.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пошук «Sheet Sander» → 1 товар; на сторінці товару є «Add to favourites»; після натискання з'явилось спливаюче повідомлення «Unauthorized, can not add product to your favorite list.» (кінцева крапка в тексті — як на demo). Знімок одразу після запиту пошуку показував проміжний (старий) список; через 1,5 с список = 1 товар.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рахунок покупця TeamB-А: INV-2026000030. Усі очікувані результати збіглися: у списку рахунків TeamB-Б його немає.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фактично: Крок 6: після введення 100 поле «Quantity» саме змінилось на 99. Крок 7: товар додано у кількості 99, лічильник кошика = 99, повідомлення «Product added to shopping cart. You can order at most 99 of this product.». Крок 8: у кошику «Combination Pliers» 99 × 14.15 = 1400.85 (очікувалось: кошик порожній). Кроки 1–4 виконано прямим переходом на сторінку товару. Значення вводилось поверх виділеного (поле при очищенні саме підставляє 1). Дефект: BUG-002.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фактично: Крок 8: після повторного додавання 5 шт. (при 99 у кошику) лічильник кошика = 104, повідомлення про межу немає. Крок 9: один рядок «Combination Pliers», Quantity 104, Total $1,471.60 (очікувалось: сумарна кількість ≤ 99). Кейс внесено до test-cases.xlsx 28.10.2026 (Бобров П.) і прорецензовано (Кочаров Д., 28.10.2026); Coverage (BL-20, F-100) оновлено. Виконано дослідницькою перевіркою до внесення кейсу; кроки 5–6 виконано як «виділити вміст поля «Quantity» і ввести 99» (у кейсі — «очистити + ввести»: порожнє поле саме підставляє 1). Для порівняння: зміна кількості в рядку кошика до 100 коректно обмежується 99 з повідомленням «You can order at most 99 of this product.». Дефект: BUG-006.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Адреса demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Браузер і версії</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вікно / режим</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Облікові записи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Примітка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://practicesoftwaretesting.com (збірка v2.5, Built 2026-10-11, Angular 20.0.5; у футері demo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27–28.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chromium 152.0.7977.167 — вбудований браузер десктопного застосунку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Windows 10/11 (NT 10.0, 64-bit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вікно 1280×800 (емуляція вікна); TC-025 — 375×812 (мобільний пресет, Android user agent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Без входу в обліковий запис (гостьовий режим); входи в акаунти не виконувались</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Відхилення від плану: у кейсах — Chrome 120+ в інкогніто, тут — Chromium 152 без інкогніто; між кейсами очищалися sessionStorage/localStorage.Дані demo скинулись між 27.10 і 28.10: каталог 59 → 50 товарів, зникли «чужі» товари за $1.99 (TC-009 повторно виконано 28.10). У TC-022 файл у поле вкладення підставлено скриптом (1024 байти), а не вікном вибору файлу ОС.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://practicesoftwaretesting.com (збірка v2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Chrome 156.0.8078.73 (Official Build, 64-bit); V8 15.6.75.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Windows 11 25H2 (Build 26200.9711)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Розмір вікна і режим інкогніто виконавцем не зафіксовано (за планом: інкогніто, 1280×800)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer@practicesoftwaretesting.com (спільний запис demo); власні записи teamb.*@example.com, створені в кейсах TC-001, TC-006, TC-029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Середовище кейсів, виконаних ІТ вручну (облікові записи, реєстрація, оформлення замовлення): TC-001…006, 019…021, 024, 026, 029. У TC-001 пароль із кейсу замінено на «Fbcdf12!» (оригінал відхилено як такий, що трапився у витоку даних).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smoke-перевірка demo перед прогоном (5.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Перевірка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Результат</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Головна сторінка відкривається, каталог показує 9 карток</t>
+  </si>
+  <si>
+    <t xml:space="preserve">так (збірка v2.5, Built 2026-10-11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пошук повертає результати; сторінка товару відкривається</t>
+  </si>
+  <si>
+    <t xml:space="preserve">так</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Додавання в кошик і крок «Cart» працюють</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Контактна форма відкривається і приймає дані</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вхід тестовим обліковим записом (customer@practicesoftwaretesting.com)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">так (TC-004, TC-019…021, TC-024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заголовок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Severity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priority</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кейс</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вимога</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reporter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Файл звіту</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кейсів у Run 1 з цим Bug ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пошук 'hammer' не знаходить «Sledgehammer»: збіг шукається не за підрядком</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Major</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-001.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кількість 100 у полі Quantity замінюється на 99, і товар додається в кошик</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GUI-30, BL-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-002.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кількість 0 замінюється на 1, і товар додається в кошик без повідомлення про діапазон</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-003.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Меню на ширині 375 px: кнопка меню 56×40, пункти меню заввишки 40 px (&lt; 44×44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-004.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Контактна форма відхиляє будь-який непорожній .txt («File should be empty.»), F-140 допускає до 1 МБ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-140, GUI-90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-005.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кошик: повторне «Add to cart» дає в рядку 104 шт. — понад межу 99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BL-20, F-100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-006.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Шапка: логотип «TOOLSHOP» замість «ШопЛайн»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trivial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GUI-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-007.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Форма реєстрації: зірочка біля обов'язкових полів стоїть непослідовно, біля «Password» її немає</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U-20, F-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-008.md</t>
+  </si>
+  <si>
     <t xml:space="preserve">BUG-009</t>
   </si>
   <si>
-    <t xml:space="preserve">Фактично: Кроки 13–14: пароль «Abcde1!» (7 символів) відхилено, але повідомлення «Password must be minimal 6 characters long.» називає межу 6 символів, що суперечить правилу «Be at least 8 characters long» на цій самій сторінці (F-10); повідомлення виведено в блоці між індикатором надійності й кнопкою «Register», а не безпосередньо під полем (GUI-50). Дефект: BUG-009.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рядок довжиною рівно 50 символів (перевірено програмно). Крок 7: форма замінилась на «Thanks for your message! We will contact you shortly.» (клас alert-success) над блоком футера; помилок немає. Це реальне надсилання на demo з тестовим email example.com.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Пошук «Sheet Sander» → 1 товар; на сторінці товару є «Add to favourites»; після натискання з'явилось спливаюче повідомлення «Unauthorized, can not add product to your favorite list.» (кінцева крапка в тексті — як на demo). Знімок одразу після запиту пошуку показував проміжний (старий) список; через 1,5 с список = 1 товар.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рахунок покупця TeamB-А: INV-2026000030. Усі очікувані результати збіглися: у списку рахунків TeamB-Б його немає.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUG-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фактично: Крок 6: після введення 100 поле «Quantity» саме змінилось на 99. Крок 7: товар додано у кількості 99, лічильник кошика = 99, повідомлення «Product added to shopping cart. You can order at most 99 of this product.». Крок 8: у кошику «Combination Pliers» 99 × 14.15 = 1400.85 (очікувалось: кошик порожній). Кроки 1–4 виконано прямим переходом на сторінку товару. Значення вводилось поверх виділеного (поле при очищенні саме підставляє 1). Дефект: BUG-002.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUG-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фактично: Крок 8: після повторного додавання 5 шт. (при 99 у кошику) лічильник кошика = 104, повідомлення про межу немає. Крок 9: один рядок «Combination Pliers», Quantity 104, Total $1,471.60 (очікувалось: сумарна кількість ≤ 99). Кейс запропоновано за результатами дослідницької перевірки (docs/sprint3/proposed-test-case-TC-031.md): його ще немає в test-cases.xlsx, потрібні рецензія і оновлення «Coverage» (BL-20, F-100). Для порівняння: зміна кількості в рядку кошика до 100 коректно обмежується 99 з повідомленням «You can order at most 99 of this product.». Дефект: BUG-006.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адреса demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Браузер і версії</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вікно / режим</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Облікові записи</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Примітка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://practicesoftwaretesting.com (збірка v2.5, Built 2026-10-11, Angular 20.0.5; у футері demo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27–28.10.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chromium 152.0.7977.167 — вбудований браузер десктопного застосунку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Windows 10/11 (NT 10.0, 64-bit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вікно 1280×800 (емуляція вікна); TC-025 — 375×812 (мобільний пресет, Android user agent)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Без входу в обліковий запис (гостьовий режим); входи в акаунти не виконувались</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Відхилення від плану: у кейсах — Chrome 120+ в інкогніто, тут — Chromium 152 без інкогніто; між кейсами очищалися sessionStorage/localStorage.Дані demo скинулись між 27.10 і 28.10: каталог 59 → 50 товарів, зникли «чужі» товари за $1.99 (TC-009 повторно виконано 28.10). У TC-022 файл у поле вкладення підставлено скриптом (1024 байти), а не вікном вибору файлу ОС.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://practicesoftwaretesting.com (збірка v2.5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28.10.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google Chrome 156.0.8078.73 (Official Build, 64-bit); V8 15.6.75.25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Windows 11 25H2 (Build 26200.9711)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Розмір вікна і режим інкогніто виконавцем не зафіксовано (за планом: інкогніто, 1280×800)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">customer@practicesoftwaretesting.com (спільний запис demo); власні записи teamb.*@example.com, створені в кейсах TC-001, TC-006, TC-029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Середовище кейсів, виконаних ІТ вручну (облікові записи, реєстрація, оформлення замовлення): TC-001…006, 019…021, 024, 026, 029. У TC-001 пароль із кейсу замінено на «Fbcdf12!» (оригінал відхилено як такий, що трапився у витоку даних).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smoke-перевірка demo перед прогоном (5.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Перевірка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Результат</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Головна сторінка відкривається, каталог показує 9 карток</t>
-  </si>
-  <si>
-    <t xml:space="preserve">так (збірка v2.5, Built 2026-10-11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.10.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Пошук повертає результати; сторінка товару відкривається</t>
-  </si>
-  <si>
-    <t xml:space="preserve">так</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Додавання в кошик і крок «Cart» працюють</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Контактна форма відкривається і приймає дані</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вхід тестовим обліковим записом (customer@practicesoftwaretesting.com)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">так (TC-004, TC-019…021, TC-024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Заголовок</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Severity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кейс</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вимога</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reporter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Файл звіту</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кейсів у Run 1 з цим Bug ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Пошук 'hammer' не знаходить «Sledgehammer»: збіг шукається не за підрядком</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Major</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-001.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кількість 100 у полі Quantity замінюється на 99, і товар додається в кошик</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GUI-30, BL-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-002.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кількість 0 замінюється на 1, і товар додається в кошик без повідомлення про діапазон</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Normal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-003.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Меню на ширині 375 px: кнопка меню 56×40, пункти меню заввишки 40 px (&lt; 44×44)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-004.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Контактна форма відхиляє будь-який непорожній .txt («File should be empty.»), F-140 допускає до 1 МБ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-140, GUI-90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-005.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кошик: повторне «Add to cart» дає в рядку 104 шт. — понад межу 99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BL-20, F-100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-006.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Шапка: логотип «TOOLSHOP» замість «ШопЛайн»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trivial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GUI-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-007.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Форма реєстрації: зірочка біля обов'язкових полів стоїть непослідовно, біля «Password» її немає</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U-20, F-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-008.md</t>
-  </si>
-  <si>
     <t xml:space="preserve">Пароль із 7 символів відхиляється повідомленням «minimal 6 characters», що суперечить правилу «мінімум 8»</t>
   </si>
   <si>
-    <t xml:space="preserve">F-10, GUI-50</t>
+    <t xml:space="preserve">F-10</t>
   </si>
   <si>
     <t xml:space="preserve">docs/sprint3/bug-reports/BUG-009.md</t>
@@ -569,6 +550,18 @@
     <t xml:space="preserve">docs/sprint3/bug-reports/BUG-013.md</t>
   </si>
   <si>
+    <t xml:space="preserve">BUG-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Реєстрація: повідомлення про помилку пароля виводиться під індикатором надійності, а не безпосередньо під полем «Password»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GUI-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/sprint3/bug-reports/BUG-014.md</t>
+  </si>
+  <si>
     <t xml:space="preserve">Спринт 3 · П1 «ШопЛайн» · Run 1 — зведення (усі значення — формули за аркушами «Run 1» і «Defects»)</t>
   </si>
   <si>
@@ -671,7 +664,7 @@
     <t xml:space="preserve">Середовища: E1 — вбудований браузер Chromium (кейси без входу в обліковий запис, 27–28.10.2026), E2 — Google Chrome (кейси з обліковими записами, 28.10.2026); деталі — на аркуші «Environment».</t>
   </si>
   <si>
-    <t xml:space="preserve">Рядок TC-031 (сірий) — запропонований кейс (див. proposed-test-case-TC-031.md), ще не внесений до test-cases.xlsx і не прорецензований.</t>
+    <t xml:space="preserve">TC-031 внесено до test-cases.xlsx 28.10.2026 і прорецензовано; виконано дослідницькою перевіркою (BUG-006).</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-011 нестабільний (1 із 2 проходжень), BUG-011 і BUG-012 без скріншотів: потребують повторного відтворення зі знімком.</t>
@@ -689,7 +682,7 @@
     <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -725,11 +718,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -808,7 +796,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -829,27 +817,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -865,11 +841,11 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -886,19 +862,11 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF1F3864"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1864,7 +1832,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
         <v>8</v>
       </c>
@@ -1988,45 +1956,45 @@
         <v>82</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
+    <row r="32" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C32" s="6" t="n">
+      <c r="C32" s="3" t="n">
         <v>46323</v>
       </c>
-      <c r="D32" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E32" s="5" t="s">
+      <c r="D32" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F32" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G32" s="5" t="s">
+      <c r="G32" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="H32" s="4" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H32"/>
   <conditionalFormatting sqref="F2:F32">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"skipped"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2043,8 +2011,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2145,7 +2112,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2231,7 +2198,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2571,10 +2538,10 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>72</v>
+        <v>156</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>138</v>
@@ -2586,7 +2553,7 @@
         <v>71</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>131</v>
@@ -2598,7 +2565,7 @@
         <v>46323</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K10" s="2" t="n">
         <f aca="false">COUNTIF('Run 1'!$G$2:$G$32,"*"&amp;A10&amp;"*")</f>
@@ -2610,7 +2577,7 @@
         <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>138</v>
@@ -2622,7 +2589,7 @@
         <v>24</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>131</v>
@@ -2634,7 +2601,7 @@
         <v>46323</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K11" s="2" t="n">
         <f aca="false">COUNTIF('Run 1'!$G$2:$G$32,"*"&amp;A11&amp;"*")</f>
@@ -2643,10 +2610,10 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>128</v>
@@ -2658,7 +2625,7 @@
         <v>53</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>131</v>
@@ -2670,7 +2637,7 @@
         <v>46323</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K12" s="2" t="n">
         <f aca="false">COUNTIF('Run 1'!$G$2:$G$32,"*"&amp;A12&amp;"*")</f>
@@ -2679,10 +2646,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>138</v>
@@ -2694,7 +2661,7 @@
         <v>53</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>131</v>
@@ -2706,7 +2673,7 @@
         <v>46323</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K13" s="2" t="n">
         <f aca="false">COUNTIF('Run 1'!$G$2:$G$32,"*"&amp;A13&amp;"*")</f>
@@ -2718,7 +2685,7 @@
         <v>59</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>134</v>
@@ -2730,7 +2697,7 @@
         <v>58</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>131</v>
@@ -2742,10 +2709,46 @@
         <v>46323</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K14" s="2" t="n">
         <f aca="false">COUNTIF('Run 1'!$G$2:$G$32,"*"&amp;A14&amp;"*")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <f aca="false">COUNTIF('Run 1'!$G$2:$G$32,"*"&amp;A15&amp;"*")</f>
         <v>1</v>
       </c>
     </row>
@@ -2775,388 +2778,388 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
+      <c r="A1" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>175</v>
+      <c r="A2" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="B3" s="12" t="n">
+      <c r="A3" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" s="9" t="n">
         <f aca="false">COUNTA('Run 1'!B2:B32)</f>
         <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="B4" s="12" t="n">
+      <c r="A4" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4" s="9" t="n">
         <f aca="false">COUNTA('Run 1'!F2:F32)</f>
         <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="B5" s="12" t="n">
+      <c r="A5" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="B5" s="9" t="n">
         <f aca="false">B3-B4</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF('Run 1'!F2:F32,"passed")</f>
         <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF('Run 1'!F2:F32,"failed")</f>
         <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="B8" s="12" t="n">
+      <c r="A8" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF('Run 1'!F2:F32,"blocked")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="B9" s="12" t="n">
+      <c r="A9" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF('Run 1'!F2:F32,"skipped")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="B10" s="12" t="n">
+      <c r="A10" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="9" t="n">
         <f aca="false">COUNTA(Defects!A2:A30)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="13"/>
+      <c r="B11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>183</v>
+      <c r="A12" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="B13" s="12" t="n">
+      <c r="A13" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B13" s="9" t="n">
         <f aca="false">COUNTIF(Defects!C2:C30,A13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>185</v>
-      </c>
-      <c r="B14" s="12" t="n">
+      <c r="A14" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B14" s="9" t="n">
         <f aca="false">COUNTIF(Defects!C2:C30,A14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="9" t="n">
         <f aca="false">COUNTIF(Defects!C2:C30,A15)</f>
         <v>3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="9" t="n">
         <f aca="false">COUNTIF(Defects!C2:C30,A16)</f>
         <v>5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="9" t="n">
         <f aca="false">COUNTIF(Defects!C2:C30,A17)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="9" t="n">
         <f aca="false">COUNTIF(Defects!C2:C30,A18)</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="B19" s="12" t="n">
+      <c r="A19" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="B19" s="9" t="n">
         <f aca="false">SUMPRODUCT(--(B13:B18&gt;0))</f>
         <v>4</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="13"/>
+      <c r="B20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>183</v>
+      <c r="A21" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>188</v>
-      </c>
-      <c r="B22" s="12" t="n">
+      <c r="A22" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B22" s="9" t="n">
         <f aca="false">COUNTIF(Defects!D2:D30,A22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>189</v>
-      </c>
-      <c r="B23" s="12" t="n">
+      <c r="A23" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B23" s="9" t="n">
         <f aca="false">COUNTIF(Defects!D2:D30,A23)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="9" t="n">
         <f aca="false">COUNTIF(Defects!D2:D30,A24)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="13"/>
+      <c r="B25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="B26" s="14" t="s">
+      <c r="A26" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>191</v>
+      <c r="C26" s="7" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="B27" s="12" t="n">
+      <c r="A27" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B27" s="9" t="n">
         <f aca="false">SUMPRODUCT(('Run 1'!F2:F32="failed")*('Run 1'!G2:G32=""))</f>
         <v>0</v>
       </c>
-      <c r="C27" s="11" t="s">
-        <v>193</v>
+      <c r="C27" s="8" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="B28" s="12" t="n">
+      <c r="A28" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B28" s="9" t="n">
         <f aca="false">SUMPRODUCT(LEN('Run 1'!G2:G32)-LEN(SUBSTITUTE('Run 1'!G2:G32,"BUG-","")))/4-SUMPRODUCT((Defects!A2:A30&lt;&gt;"")*COUNTIF('Run 1'!G2:G32,"*"&amp;Defects!A2:A30&amp;"*"))</f>
         <v>0</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>193</v>
+      <c r="C28" s="8" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="B29" s="12" t="n">
+      <c r="A29" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="B29" s="9" t="n">
         <f aca="false">SUMPRODUCT((Defects!A2:A30&lt;&gt;"")*(COUNTIF('Run 1'!G2:G32,"*"&amp;Defects!A2:A30&amp;"*")=0))</f>
         <v>0</v>
       </c>
-      <c r="C29" s="11" t="s">
-        <v>193</v>
+      <c r="C29" s="8" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="B30" s="12" t="n">
+      <c r="A30" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B30" s="9" t="n">
         <f aca="false">SUMPRODUCT(('Run 1'!F2:F32="blocked")*('Run 1'!H2:H32=""))</f>
         <v>0</v>
       </c>
-      <c r="C30" s="11" t="s">
-        <v>193</v>
+      <c r="C30" s="8" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="B31" s="12" t="n">
+      <c r="A31" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B31" s="9" t="n">
         <f aca="false">SUMPRODUCT(('Run 1'!F2:F32&lt;&gt;"")*(('Run 1'!C2:C32="")+('Run 1'!D2:D32="")&gt;0))</f>
         <v>0</v>
       </c>
-      <c r="C31" s="11" t="s">
-        <v>193</v>
+      <c r="C31" s="8" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="13"/>
+      <c r="B32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="C33" s="10" t="s">
+      <c r="A33" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>200</v>
+      <c r="D33" s="7" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="B34" s="12" t="n">
+      <c r="A34" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B34" s="9" t="n">
         <f aca="false">B3</f>
         <v>31</v>
       </c>
-      <c r="C34" s="11" t="n">
+      <c r="C34" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="D34" s="11" t="str">
+      <c r="D34" s="8" t="str">
         <f aca="false">IF(B34&gt;=C34,"виконано","бракує "&amp;(C34-B34))</f>
         <v>виконано</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
-        <v>202</v>
-      </c>
-      <c r="B35" s="12" t="n">
+      <c r="A35" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="B35" s="9" t="n">
         <f aca="false">B10</f>
-        <v>13</v>
-      </c>
-      <c r="C35" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="D35" s="11" t="str">
+        <v>14</v>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="8" t="str">
         <f aca="false">IF(B35&gt;=C35,"виконано","бракує "&amp;(C35-B35))</f>
         <v>виконано</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="B36" s="12" t="n">
+      <c r="A36" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B36" s="9" t="n">
         <f aca="false">B19</f>
         <v>4</v>
       </c>
-      <c r="C36" s="11" t="n">
+      <c r="C36" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D36" s="11" t="str">
+      <c r="D36" s="8" t="str">
         <f aca="false">IF(B36&gt;=C36,"виконано","бракує "&amp;(C36-B36))</f>
         <v>виконано</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="s">
-        <v>204</v>
+      <c r="A38" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16" t="s">
-        <v>205</v>
-      </c>
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
+      <c r="A39" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="16" t="s">
-        <v>206</v>
-      </c>
-      <c r="B40" s="16"/>
-      <c r="C40" s="16"/>
-      <c r="D40" s="16"/>
+      <c r="A40" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
     </row>
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="B41" s="16"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="16"/>
+      <c r="A41" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="B42" s="16"/>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
+      <c r="A42" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="16"/>
+      <c r="A43" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>